<commit_message>
AGREGADO_COSTOS - reportes - sesionesActivas
</commit_message>
<xml_diff>
--- a/TomaInventarioWEB/Plantillas/Plantilla_Producto.xlsx
+++ b/TomaInventarioWEB/Plantillas/Plantilla_Producto.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\User\Desktop\Documentos\TomaDeInventario - Web\TomaInventario-GitHub\TomaInventarioWEB\Plantillas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmspe\Downloads\Toma_Inventario-GitHub\TomaInventarioWEB\TomaInventarioWEB\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70048BB1-1388-428E-BF96-9DCA34810A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9E8042B-3695-42F5-9FE4-4D162DB33A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1320" windowWidth="26085" windowHeight="14160" xr2:uid="{67C386F5-27F8-4261-BF4C-5F77FEEA6F00}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{67C386F5-27F8-4261-BF4C-5F77FEEA6F00}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>CPU MC9090K</t>
   </si>
@@ -64,13 +64,22 @@
   </si>
   <si>
     <t>COD_UNIDAD_MEDIDA</t>
+  </si>
+  <si>
+    <t>PRECIO_COSTO</t>
+  </si>
+  <si>
+    <t>COD_MONEDA</t>
+  </si>
+  <si>
+    <t>USD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -99,6 +108,14 @@
       <color theme="0"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -190,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -206,6 +223,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -530,18 +554,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51F00432-D8BC-42FC-B196-DFEFADEB5870}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="80.140625" customWidth="1"/>
     <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" style="7" customWidth="1"/>
-    <col min="7" max="7" width="46.85546875" style="7" customWidth="1"/>
+    <col min="4" max="4" width="34.85546875" customWidth="1"/>
+    <col min="5" max="5" width="36.42578125" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" style="7" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" style="7" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" style="7" customWidth="1"/>
+    <col min="9" max="9" width="11.85546875" customWidth="1"/>
+    <col min="10" max="10" width="21.140625" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" customWidth="1"/>
+    <col min="12" max="12" width="24.42578125" customWidth="1"/>
+    <col min="13" max="13" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>7</v>
       </c>
@@ -551,13 +582,19 @@
       <c r="C1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="D1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="9"/>
-      <c r="H1" s="10"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="13"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -567,26 +604,39 @@
       <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="D2" s="10">
+        <v>1730.2</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K8" s="8"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="K1:M1"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="AVISO!" error="No puede Ingresar más de 20 caracteres en esta celda" sqref="A1:A1048576" xr:uid="{5634BA0D-829E-488E-AF26-19ABDA1CB07C}">
       <formula1>20</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="AVISO!" error="No puede ingresar más de 200 caracteres en esta celda" sqref="B1:B1048576 C1:C2" xr:uid="{B078B425-461D-4E96-AE7F-85715965BEFD}">
+    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="AVISO!" error="No puede ingresar más de 200 caracteres en esta celda" sqref="B1:B1048576 C1:E2" xr:uid="{B078B425-461D-4E96-AE7F-85715965BEFD}">
       <formula1>200</formula1>
     </dataValidation>
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H6:H1048576 H3" xr:uid="{6AFC20A7-5642-4747-A22E-B9079618770F}">

</xml_diff>